<commit_message>
Metadata of new covariate stack JORD
</commit_message>
<xml_diff>
--- a/covariates_overview_20260626.xlsx
+++ b/covariates_overview_20260626.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au802520_uni_au_dk/Documents/PhD/AU_DSM_meta/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au704633_uni_au_dk/Documents/Documents/AARHUS_PhD/DSMactivities/Repos/AU_DSM_metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="8_{8D936188-1850-4E56-89C0-09BF28A24A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58871820-B477-456E-976B-AA2982797E08}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{8D936188-1850-4E56-89C0-09BF28A24A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74827480-37AC-493D-8E46-5969CE6301FC}"/>
   <bookViews>
-    <workbookView xWindow="47895" yWindow="-13560" windowWidth="19410" windowHeight="20985" xr2:uid="{2BA01098-D2FC-417D-8769-17E5D0886F88}"/>
+    <workbookView xWindow="38280" yWindow="-1815" windowWidth="29040" windowHeight="15720" xr2:uid="{2BA01098-D2FC-417D-8769-17E5D0886F88}"/>
   </bookViews>
   <sheets>
     <sheet name="covariates_overview_20260317" sheetId="1" r:id="rId1"/>
@@ -3196,10 +3196,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3518,26 +3514,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EBDCFF0-81C6-428C-9378-5565086C0D01}">
   <dimension ref="A1:T266"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="66.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="66.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" customWidth="1"/>
-    <col min="4" max="4" width="15.6328125" customWidth="1"/>
-    <col min="5" max="5" width="18.453125" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="82.54296875" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="82.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" customWidth="1"/>
     <col min="9" max="9" width="23" customWidth="1"/>
-    <col min="10" max="10" width="67.54296875" customWidth="1"/>
-    <col min="11" max="12" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="37.08984375" customWidth="1"/>
-    <col min="14" max="14" width="16.90625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="67.5703125" customWidth="1"/>
+    <col min="11" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="37.140625" customWidth="1"/>
+    <col min="14" max="14" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>543</v>
       </c>
@@ -3587,7 +3583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>542</v>
       </c>
@@ -3637,7 +3633,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>553</v>
       </c>
@@ -3687,7 +3683,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>554</v>
       </c>
@@ -3737,7 +3733,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>555</v>
       </c>
@@ -3787,7 +3783,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>544</v>
       </c>
@@ -3837,7 +3833,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>545</v>
       </c>
@@ -3887,7 +3883,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>546</v>
       </c>
@@ -3937,7 +3933,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>547</v>
       </c>
@@ -3987,7 +3983,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>548</v>
       </c>
@@ -4037,7 +4033,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>549</v>
       </c>
@@ -4087,7 +4083,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>550</v>
       </c>
@@ -4137,7 +4133,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>551</v>
       </c>
@@ -4187,7 +4183,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>552</v>
       </c>
@@ -4237,7 +4233,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>556</v>
       </c>
@@ -4287,7 +4283,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>557</v>
       </c>
@@ -4337,7 +4333,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>558</v>
       </c>
@@ -4387,7 +4383,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>559</v>
       </c>
@@ -4437,7 +4433,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>560</v>
       </c>
@@ -4487,7 +4483,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>561</v>
       </c>
@@ -4537,7 +4533,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>562</v>
       </c>
@@ -4587,7 +4583,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>563</v>
       </c>
@@ -4637,7 +4633,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>564</v>
       </c>
@@ -4687,7 +4683,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>565</v>
       </c>
@@ -4737,7 +4733,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>566</v>
       </c>
@@ -4787,7 +4783,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>567</v>
       </c>
@@ -4837,7 +4833,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>570</v>
       </c>
@@ -4888,7 +4884,7 @@
       </c>
       <c r="T27" s="1"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>571</v>
       </c>
@@ -4938,7 +4934,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>574</v>
       </c>
@@ -4985,7 +4981,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>568</v>
       </c>
@@ -5035,7 +5031,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>575</v>
       </c>
@@ -5082,7 +5078,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>572</v>
       </c>
@@ -5132,7 +5128,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>569</v>
       </c>
@@ -5182,7 +5178,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>573</v>
       </c>
@@ -5232,7 +5228,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>579</v>
       </c>
@@ -5282,7 +5278,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>580</v>
       </c>
@@ -5332,7 +5328,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>581</v>
       </c>
@@ -5382,7 +5378,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>582</v>
       </c>
@@ -5432,7 +5428,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>583</v>
       </c>
@@ -5482,7 +5478,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>584</v>
       </c>
@@ -5532,7 +5528,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>585</v>
       </c>
@@ -5582,7 +5578,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>586</v>
       </c>
@@ -5632,7 +5628,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>587</v>
       </c>
@@ -5682,7 +5678,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>588</v>
       </c>
@@ -5732,7 +5728,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>589</v>
       </c>
@@ -5782,7 +5778,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>590</v>
       </c>
@@ -5832,7 +5828,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>591</v>
       </c>
@@ -5882,7 +5878,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>592</v>
       </c>
@@ -5932,7 +5928,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>593</v>
       </c>
@@ -5982,7 +5978,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>594</v>
       </c>
@@ -6032,7 +6028,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>595</v>
       </c>
@@ -6082,7 +6078,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>596</v>
       </c>
@@ -6132,7 +6128,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>597</v>
       </c>
@@ -6182,7 +6178,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>598</v>
       </c>
@@ -6232,7 +6228,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>599</v>
       </c>
@@ -6282,7 +6278,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>600</v>
       </c>
@@ -6332,7 +6328,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>601</v>
       </c>
@@ -6382,7 +6378,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>602</v>
       </c>
@@ -6432,7 +6428,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>603</v>
       </c>
@@ -6482,7 +6478,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>604</v>
       </c>
@@ -6532,7 +6528,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>605</v>
       </c>
@@ -6582,7 +6578,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>606</v>
       </c>
@@ -6632,7 +6628,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>607</v>
       </c>
@@ -6682,7 +6678,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>608</v>
       </c>
@@ -6732,7 +6728,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>609</v>
       </c>
@@ -6782,7 +6778,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>610</v>
       </c>
@@ -6832,7 +6828,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>611</v>
       </c>
@@ -6882,7 +6878,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>612</v>
       </c>
@@ -6932,7 +6928,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>613</v>
       </c>
@@ -6982,7 +6978,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>614</v>
       </c>
@@ -7032,7 +7028,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>615</v>
       </c>
@@ -7082,7 +7078,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>616</v>
       </c>
@@ -7132,7 +7128,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>617</v>
       </c>
@@ -7182,7 +7178,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>618</v>
       </c>
@@ -7232,7 +7228,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>619</v>
       </c>
@@ -7282,7 +7278,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>620</v>
       </c>
@@ -7332,7 +7328,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>621</v>
       </c>
@@ -7382,7 +7378,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>622</v>
       </c>
@@ -7432,7 +7428,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>623</v>
       </c>
@@ -7482,7 +7478,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>624</v>
       </c>
@@ -7532,7 +7528,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>625</v>
       </c>
@@ -7582,7 +7578,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>626</v>
       </c>
@@ -7632,7 +7628,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>627</v>
       </c>
@@ -7682,7 +7678,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>628</v>
       </c>
@@ -7732,7 +7728,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>629</v>
       </c>
@@ -7782,7 +7778,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>630</v>
       </c>
@@ -7832,7 +7828,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>631</v>
       </c>
@@ -7882,7 +7878,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>632</v>
       </c>
@@ -7932,7 +7928,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>633</v>
       </c>
@@ -7982,7 +7978,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>634</v>
       </c>
@@ -8032,7 +8028,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>635</v>
       </c>
@@ -8082,7 +8078,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>636</v>
       </c>
@@ -8132,7 +8128,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>637</v>
       </c>
@@ -8182,7 +8178,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>638</v>
       </c>
@@ -8232,7 +8228,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>639</v>
       </c>
@@ -8282,7 +8278,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>640</v>
       </c>
@@ -8332,7 +8328,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>641</v>
       </c>
@@ -8382,7 +8378,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>576</v>
       </c>
@@ -8432,7 +8428,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>642</v>
       </c>
@@ -8482,7 +8478,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>643</v>
       </c>
@@ -8532,7 +8528,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>577</v>
       </c>
@@ -8582,7 +8578,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>644</v>
       </c>
@@ -8632,7 +8628,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>645</v>
       </c>
@@ -8682,7 +8678,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>646</v>
       </c>
@@ -8732,7 +8728,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>647</v>
       </c>
@@ -8782,7 +8778,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>648</v>
       </c>
@@ -8832,7 +8828,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>649</v>
       </c>
@@ -8882,7 +8878,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>650</v>
       </c>
@@ -8932,7 +8928,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>651</v>
       </c>
@@ -8982,7 +8978,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>652</v>
       </c>
@@ -9032,7 +9028,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>653</v>
       </c>
@@ -9082,7 +9078,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>654</v>
       </c>
@@ -9132,7 +9128,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>578</v>
       </c>
@@ -9182,7 +9178,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>655</v>
       </c>
@@ -9229,7 +9225,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>656</v>
       </c>
@@ -9276,7 +9272,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>657</v>
       </c>
@@ -9323,7 +9319,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>658</v>
       </c>
@@ -9370,7 +9366,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>659</v>
       </c>
@@ -9417,7 +9413,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>660</v>
       </c>
@@ -9464,7 +9460,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>661</v>
       </c>
@@ -9511,7 +9507,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>662</v>
       </c>
@@ -9558,7 +9554,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>663</v>
       </c>
@@ -9605,7 +9601,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>664</v>
       </c>
@@ -9652,7 +9648,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>665</v>
       </c>
@@ -9699,7 +9695,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>666</v>
       </c>
@@ -9746,7 +9742,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>667</v>
       </c>
@@ -9796,7 +9792,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>668</v>
       </c>
@@ -9846,7 +9842,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>669</v>
       </c>
@@ -9896,7 +9892,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>670</v>
       </c>
@@ -9946,7 +9942,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>671</v>
       </c>
@@ -9996,7 +9992,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>672</v>
       </c>
@@ -10043,7 +10039,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>673</v>
       </c>
@@ -10090,7 +10086,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>674</v>
       </c>
@@ -10137,7 +10133,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>675</v>
       </c>
@@ -10184,7 +10180,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>676</v>
       </c>
@@ -10231,7 +10227,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>677</v>
       </c>
@@ -10278,7 +10274,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>678</v>
       </c>
@@ -10325,7 +10321,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>679</v>
       </c>
@@ -10372,7 +10368,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>680</v>
       </c>
@@ -10419,7 +10415,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>681</v>
       </c>
@@ -10466,7 +10462,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>682</v>
       </c>
@@ -10513,7 +10509,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>683</v>
       </c>
@@ -10560,7 +10556,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>684</v>
       </c>
@@ -10607,7 +10603,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>685</v>
       </c>
@@ -10654,7 +10650,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>686</v>
       </c>
@@ -10701,7 +10697,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>687</v>
       </c>
@@ -10748,7 +10744,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>688</v>
       </c>
@@ -10795,7 +10791,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>689</v>
       </c>
@@ -10842,7 +10838,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>690</v>
       </c>
@@ -10889,7 +10885,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>691</v>
       </c>
@@ -10936,7 +10932,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>692</v>
       </c>
@@ -10983,7 +10979,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>693</v>
       </c>
@@ -11030,7 +11026,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>694</v>
       </c>
@@ -11077,7 +11073,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>695</v>
       </c>
@@ -11124,7 +11120,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>696</v>
       </c>
@@ -11171,7 +11167,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>697</v>
       </c>
@@ -11218,7 +11214,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>698</v>
       </c>
@@ -11265,7 +11261,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>699</v>
       </c>
@@ -11312,7 +11308,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>700</v>
       </c>
@@ -11359,7 +11355,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>701</v>
       </c>
@@ -11406,7 +11402,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>702</v>
       </c>
@@ -11453,7 +11449,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>703</v>
       </c>
@@ -11500,7 +11496,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>704</v>
       </c>
@@ -11547,7 +11543,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>705</v>
       </c>
@@ -11594,7 +11590,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>706</v>
       </c>
@@ -11641,7 +11637,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>707</v>
       </c>
@@ -11688,7 +11684,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>708</v>
       </c>
@@ -11735,7 +11731,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>709</v>
       </c>
@@ -11782,7 +11778,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>710</v>
       </c>
@@ -11829,7 +11825,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>711</v>
       </c>
@@ -11876,7 +11872,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>712</v>
       </c>
@@ -11923,7 +11919,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>713</v>
       </c>
@@ -11970,7 +11966,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>714</v>
       </c>
@@ -12017,7 +12013,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>715</v>
       </c>
@@ -12064,7 +12060,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>716</v>
       </c>
@@ -12111,7 +12107,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>717</v>
       </c>
@@ -12158,7 +12154,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>718</v>
       </c>
@@ -12205,7 +12201,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>719</v>
       </c>
@@ -12252,7 +12248,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>720</v>
       </c>
@@ -12299,7 +12295,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>721</v>
       </c>
@@ -12346,7 +12342,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>722</v>
       </c>
@@ -12393,7 +12389,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>723</v>
       </c>
@@ -12440,7 +12436,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>724</v>
       </c>
@@ -12487,7 +12483,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>725</v>
       </c>
@@ -12534,7 +12530,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>726</v>
       </c>
@@ -12581,7 +12577,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>727</v>
       </c>
@@ -12628,7 +12624,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>728</v>
       </c>
@@ -12675,7 +12671,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>729</v>
       </c>
@@ -12722,7 +12718,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>730</v>
       </c>
@@ -12769,7 +12765,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>731</v>
       </c>
@@ -12816,7 +12812,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>732</v>
       </c>
@@ -12863,7 +12859,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>733</v>
       </c>
@@ -12910,7 +12906,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>734</v>
       </c>
@@ -12957,7 +12953,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>735</v>
       </c>
@@ -13004,7 +13000,7 @@
         <v>45355</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>736</v>
       </c>
@@ -13054,7 +13050,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>737</v>
       </c>
@@ -13104,7 +13100,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>738</v>
       </c>
@@ -13154,7 +13150,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>739</v>
       </c>
@@ -13204,7 +13200,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>740</v>
       </c>
@@ -13254,7 +13250,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>741</v>
       </c>
@@ -13304,7 +13300,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>742</v>
       </c>
@@ -13354,7 +13350,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>743</v>
       </c>
@@ -13404,7 +13400,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>744</v>
       </c>
@@ -13454,7 +13450,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>745</v>
       </c>
@@ -13504,7 +13500,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>746</v>
       </c>
@@ -13554,7 +13550,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>747</v>
       </c>
@@ -13604,7 +13600,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>748</v>
       </c>
@@ -13654,7 +13650,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>749</v>
       </c>
@@ -13704,7 +13700,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>750</v>
       </c>
@@ -13754,7 +13750,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>751</v>
       </c>
@@ -13804,7 +13800,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>752</v>
       </c>
@@ -13854,7 +13850,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>753</v>
       </c>
@@ -13904,7 +13900,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>754</v>
       </c>
@@ -13954,7 +13950,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>755</v>
       </c>
@@ -14004,7 +14000,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>756</v>
       </c>
@@ -14054,7 +14050,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>757</v>
       </c>
@@ -14104,7 +14100,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>758</v>
       </c>
@@ -14154,7 +14150,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>759</v>
       </c>
@@ -14204,7 +14200,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>760</v>
       </c>
@@ -14254,7 +14250,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>761</v>
       </c>
@@ -14304,7 +14300,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>762</v>
       </c>
@@ -14354,7 +14350,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>763</v>
       </c>
@@ -14404,7 +14400,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>764</v>
       </c>
@@ -14454,7 +14450,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>765</v>
       </c>
@@ -14504,7 +14500,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>766</v>
       </c>
@@ -14554,7 +14550,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>767</v>
       </c>
@@ -14604,7 +14600,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>768</v>
       </c>
@@ -14654,7 +14650,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>769</v>
       </c>
@@ -14704,7 +14700,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>770</v>
       </c>
@@ -14754,7 +14750,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>771</v>
       </c>
@@ -14804,7 +14800,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>772</v>
       </c>
@@ -14854,7 +14850,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>773</v>
       </c>
@@ -14904,7 +14900,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>774</v>
       </c>
@@ -14954,7 +14950,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>775</v>
       </c>
@@ -15004,7 +15000,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>776</v>
       </c>
@@ -15054,7 +15050,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>777</v>
       </c>
@@ -15104,7 +15100,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>778</v>
       </c>
@@ -15154,7 +15150,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>779</v>
       </c>
@@ -15204,7 +15200,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>780</v>
       </c>
@@ -15254,7 +15250,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>781</v>
       </c>
@@ -15304,7 +15300,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>782</v>
       </c>
@@ -15354,7 +15350,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>783</v>
       </c>
@@ -15404,7 +15400,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>784</v>
       </c>
@@ -15454,7 +15450,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>785</v>
       </c>
@@ -15504,7 +15500,7 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>786</v>
       </c>
@@ -15554,7 +15550,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>787</v>
       </c>
@@ -15604,7 +15600,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>788</v>
       </c>
@@ -15648,7 +15644,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>789</v>
       </c>
@@ -15692,7 +15688,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>790</v>
       </c>
@@ -15736,7 +15732,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>791</v>
       </c>
@@ -15780,7 +15776,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>792</v>
       </c>
@@ -15824,7 +15820,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>793</v>
       </c>
@@ -15868,7 +15864,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>794</v>
       </c>
@@ -15912,7 +15908,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>795</v>
       </c>
@@ -15962,7 +15958,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>796</v>
       </c>
@@ -16012,7 +16008,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>797</v>
       </c>
@@ -16062,7 +16058,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="257" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>798</v>
       </c>
@@ -16112,7 +16108,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>799</v>
       </c>
@@ -16162,7 +16158,7 @@
         <v>44824</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>837</v>
       </c>
@@ -16209,7 +16205,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="260" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>838</v>
       </c>
@@ -16256,7 +16252,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>839</v>
       </c>
@@ -16303,7 +16299,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>840</v>
       </c>
@@ -16350,7 +16346,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>859</v>
       </c>
@@ -16391,7 +16387,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>860</v>
       </c>
@@ -16432,7 +16428,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>861</v>
       </c>
@@ -16473,7 +16469,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="266" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>862</v>
       </c>

</xml_diff>